<commit_message>
Midway backup, after some very important updates in Stock_trading_processes.docx
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Sample_Result_Mapped_Expired_OrderBook_Equity.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Sample_Result_Mapped_Expired_OrderBook_Equity.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\order_files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\PENDING_ORDERS_REPOSITORY_FILES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99874A93-53DA-47E4-9E6F-D430BC0D0AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4E261BD-6F3A-4012-82FB-2B67672FC2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7687,7 +7687,7 @@
         <v>1424</v>
       </c>
       <c r="F194">
-        <f t="shared" ref="F194:F257" si="6">((E194-H194)/H194)*100</f>
+        <f t="shared" ref="F194:F218" si="6">((E194-H194)/H194)*100</f>
         <v>7.0676691729323311</v>
       </c>
       <c r="G194" s="12" t="s">
@@ -11656,7 +11656,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14BC8B01-30D9-4196-92E7-1F70C7F62A69}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:H198"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -12234,7 +12233,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>102</v>
       </c>
@@ -12263,7 +12262,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>111</v>
       </c>
@@ -12466,7 +12465,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>113</v>
       </c>
@@ -12524,7 +12523,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>102</v>
       </c>
@@ -12553,7 +12552,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>108</v>
       </c>
@@ -12582,7 +12581,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>105</v>
       </c>
@@ -12669,7 +12668,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>115</v>
       </c>
@@ -12756,7 +12755,7 @@
         <v>NO MATCH IN TARGET</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>117</v>
       </c>
@@ -12930,7 +12929,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>120</v>
       </c>
@@ -13017,7 +13016,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>118</v>
       </c>
@@ -13046,7 +13045,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>122</v>
       </c>
@@ -13104,7 +13103,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>108</v>
       </c>
@@ -13191,7 +13190,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>108</v>
       </c>
@@ -13220,7 +13219,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>123</v>
       </c>
@@ -13249,7 +13248,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>111</v>
       </c>
@@ -13278,7 +13277,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>109</v>
       </c>
@@ -13307,7 +13306,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>124</v>
       </c>
@@ -13336,7 +13335,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>120</v>
       </c>
@@ -13394,7 +13393,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>117</v>
       </c>
@@ -13423,7 +13422,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>111</v>
       </c>
@@ -13452,7 +13451,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>108</v>
       </c>
@@ -13568,7 +13567,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>108</v>
       </c>
@@ -13597,7 +13596,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>108</v>
       </c>
@@ -13684,7 +13683,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>123</v>
       </c>
@@ -13713,7 +13712,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>116</v>
       </c>
@@ -13742,7 +13741,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>124</v>
       </c>
@@ -13771,7 +13770,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>125</v>
       </c>
@@ -13829,7 +13828,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>124</v>
       </c>
@@ -13858,7 +13857,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>127</v>
       </c>
@@ -13916,7 +13915,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>117</v>
       </c>
@@ -13945,7 +13944,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>128</v>
       </c>
@@ -14003,7 +14002,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>124</v>
       </c>
@@ -14032,7 +14031,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>122</v>
       </c>
@@ -14061,7 +14060,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>120</v>
       </c>
@@ -14119,7 +14118,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>129</v>
       </c>
@@ -14148,7 +14147,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>130</v>
       </c>
@@ -14177,7 +14176,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>124</v>
       </c>
@@ -14206,7 +14205,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>131</v>
       </c>
@@ -14235,7 +14234,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>102</v>
       </c>
@@ -14264,7 +14263,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>122</v>
       </c>
@@ -14293,7 +14292,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>117</v>
       </c>
@@ -14322,7 +14321,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>120</v>
       </c>
@@ -14351,7 +14350,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>122</v>
       </c>
@@ -14380,7 +14379,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>109</v>
       </c>
@@ -14409,7 +14408,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>124</v>
       </c>
@@ -14438,7 +14437,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>127</v>
       </c>
@@ -14467,7 +14466,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>132</v>
       </c>
@@ -14496,7 +14495,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>109</v>
       </c>
@@ -14525,7 +14524,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>130</v>
       </c>
@@ -14554,7 +14553,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>125</v>
       </c>
@@ -14612,7 +14611,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
         <v>122</v>
       </c>
@@ -14641,7 +14640,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
         <v>108</v>
       </c>
@@ -14670,7 +14669,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
         <v>108</v>
       </c>
@@ -14728,7 +14727,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
         <v>124</v>
       </c>
@@ -14757,7 +14756,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
         <v>133</v>
       </c>
@@ -14786,7 +14785,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
         <v>111</v>
       </c>
@@ -14815,7 +14814,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
         <v>134</v>
       </c>
@@ -14844,7 +14843,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
         <v>135</v>
       </c>
@@ -14902,7 +14901,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
         <v>136</v>
       </c>
@@ -14960,7 +14959,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
         <v>134</v>
       </c>
@@ -14989,7 +14988,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
         <v>120</v>
       </c>
@@ -15018,7 +15017,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
         <v>133</v>
       </c>
@@ -15047,7 +15046,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
         <v>137</v>
       </c>
@@ -15076,7 +15075,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
         <v>109</v>
       </c>
@@ -15105,7 +15104,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
         <v>135</v>
       </c>
@@ -15134,7 +15133,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
         <v>134</v>
       </c>
@@ -15163,7 +15162,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
         <v>120</v>
       </c>
@@ -15192,7 +15191,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
         <v>113</v>
       </c>
@@ -15221,7 +15220,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
         <v>116</v>
       </c>
@@ -15250,7 +15249,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
         <v>123</v>
       </c>
@@ -15279,7 +15278,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
         <v>138</v>
       </c>
@@ -15308,7 +15307,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
         <v>137</v>
       </c>
@@ -15337,7 +15336,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
         <v>137</v>
       </c>
@@ -15366,7 +15365,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
         <v>139</v>
       </c>
@@ -15395,7 +15394,7 @@
         <v>NO MATCH IN TARGET</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
         <v>134</v>
       </c>
@@ -15424,7 +15423,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
         <v>134</v>
       </c>
@@ -15453,7 +15452,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
         <v>114</v>
       </c>
@@ -15482,7 +15481,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
         <v>114</v>
       </c>
@@ -15511,7 +15510,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
         <v>122</v>
       </c>
@@ -15540,7 +15539,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
         <v>138</v>
       </c>
@@ -15569,7 +15568,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
         <v>137</v>
       </c>
@@ -15598,7 +15597,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
         <v>131</v>
       </c>
@@ -15627,7 +15626,7 @@
         <v>NO MATCH IN TARGET</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
         <v>140</v>
       </c>
@@ -15656,7 +15655,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
         <v>120</v>
       </c>
@@ -15743,7 +15742,7 @@
         <v>NO MATCH IN TARGET</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
         <v>111</v>
       </c>
@@ -15772,7 +15771,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" t="s">
         <v>133</v>
       </c>
@@ -15801,7 +15800,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A144" t="s">
         <v>136</v>
       </c>
@@ -15830,7 +15829,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" t="s">
         <v>109</v>
       </c>
@@ -15888,7 +15887,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" t="s">
         <v>138</v>
       </c>
@@ -15917,7 +15916,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" t="s">
         <v>130</v>
       </c>
@@ -15946,7 +15945,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A149" t="s">
         <v>138</v>
       </c>
@@ -16004,7 +16003,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A151" t="s">
         <v>127</v>
       </c>
@@ -16033,7 +16032,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A152" t="s">
         <v>132</v>
       </c>
@@ -16091,7 +16090,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A154" t="s">
         <v>108</v>
       </c>
@@ -16149,7 +16148,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" t="s">
         <v>120</v>
       </c>
@@ -16178,7 +16177,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A157" t="s">
         <v>122</v>
       </c>
@@ -16207,7 +16206,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A158" t="s">
         <v>141</v>
       </c>
@@ -16236,7 +16235,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A159" t="s">
         <v>130</v>
       </c>
@@ -16265,7 +16264,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A160" t="s">
         <v>111</v>
       </c>
@@ -16294,7 +16293,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A161" t="s">
         <v>120</v>
       </c>
@@ -16352,7 +16351,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A163" t="s">
         <v>111</v>
       </c>
@@ -16410,7 +16409,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A165" t="s">
         <v>127</v>
       </c>
@@ -16468,7 +16467,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A167" t="s">
         <v>117</v>
       </c>
@@ -16497,7 +16496,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A168" t="s">
         <v>122</v>
       </c>
@@ -16526,7 +16525,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A169" t="s">
         <v>143</v>
       </c>
@@ -16584,7 +16583,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A171" t="s">
         <v>120</v>
       </c>
@@ -16613,7 +16612,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A172" t="s">
         <v>109</v>
       </c>
@@ -16642,7 +16641,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="173" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A173" t="s">
         <v>143</v>
       </c>
@@ -16671,7 +16670,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="174" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A174" t="s">
         <v>132</v>
       </c>
@@ -16729,7 +16728,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="176" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A176" s="5" t="s">
         <v>146</v>
       </c>
@@ -16758,7 +16757,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A177" s="5" t="s">
         <v>127</v>
       </c>
@@ -16816,7 +16815,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="179" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A179" s="5" t="s">
         <v>124</v>
       </c>
@@ -16845,7 +16844,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A180" s="5" t="s">
         <v>124</v>
       </c>
@@ -16874,7 +16873,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="181" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="181" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A181" s="5" t="s">
         <v>146</v>
       </c>
@@ -16903,7 +16902,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="182" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A182" s="5" t="s">
         <v>143</v>
       </c>
@@ -17106,7 +17105,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="189" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A189" s="5" t="s">
         <v>150</v>
       </c>
@@ -17338,7 +17337,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A197" s="1">
         <v>46234.6875</v>
       </c>
@@ -17367,7 +17366,7 @@
         <v>MATCHED</v>
       </c>
     </row>
-    <row r="198" spans="1:8" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="198" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A198" t="s">
         <v>111</v>
       </c>
@@ -17397,13 +17396,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="H1:H198" xr:uid="{14BC8B01-30D9-4196-92E7-1F70C7F62A69}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="NO MATCH IN TARGET"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>